<commit_message>
Giới thiệu đề tài, Giai đoạn 1
</commit_message>
<xml_diff>
--- a/docs/intro.xlsx
+++ b/docs/intro.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATN_NGUYEN_CHI_THANH\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C8B0520-4757-450D-96CB-CE3CFE22AC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955AA1AA-8CE6-476C-A86E-54F27EFF7CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Họ tên</t>
   </si>
@@ -43,6 +43,28 @@
   </si>
   <si>
     <t>Nguyễn Chí Thành</t>
+  </si>
+  <si>
+    <t>Website: Cửa hàng tạp hóa trực tuyến</t>
+  </si>
+  <si>
+    <t>Đề tài xây dựng website bán hàng tạp hóa trực tuyến nhằm hỗ trợ người dùng có thể dễ dàng tìm kiếm, lựa chọn và mua sắm các sản phẩm thiết yếu hằng ngày ngay tại nhà. Hệ thống giúp cửa hàng quản lý sản phẩm, đơn hàng và khách hàng một cách hiệu quả, đồng thời mang đến trải nghiệm mua sắm tiện lợi, tiết kiệm thời gian cho người tiêu dùng.</t>
+  </si>
+  <si>
+    <t>1. Đối với khách hàng:
++ Đăng ký, đăng nhập và quản lý tài khoản cá nhân.
++ Tìm kiếm và xem chi tiết sản phẩm (theo danh mục, từ khóa).
++ Thêm sản phẩm vào giỏ hàng, cập nhật số lượng, xóa sản phẩm.
++ Đặt hàng và lựa chọn phương thức thanh toán.
++ Theo dõi trạng thái đơn hàng.
++ Đánh giá và phản hồi về sản phẩm.
++ Nói chuyện với Chatbot Ai để tư vấn sản phẩm.
+2. Đối với quản trị viên (Admin):
++ Quản lý danh mục và sản phẩm (thêm, sửa, xóa, cập nhật tồn kho).
++ Quản lý tài khoản khách hàng.
++ Quản lý đơn hàng (xác nhận, xử lý, hủy, giao hàng).
++ Quản lý tin tức, khuyến mãi.
++ Thống kê doanh thu, báo cáo bán hàng bằng biểu đồ.</t>
   </si>
 </sst>
 </file>
@@ -382,15 +404,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="46.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="18.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="46.1796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -398,7 +420,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -406,23 +428,29 @@
         <v>191667</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="61.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" ht="137.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="137.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" ht="114.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Báo cáo tuần 8
</commit_message>
<xml_diff>
--- a/docs/intro.xlsx
+++ b/docs/intro.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATN_NGUYEN_CHI_THANH\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7BD845-84F1-4728-9775-9275840223A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C661A4C8-AC7C-4E9B-9F14-3DBD9CEAAAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>